<commit_message>
docs(exports): regenerate Office files with W5 backfill feature
Architecture.docx (spec ingestion note + Sprint 3), Study-Plans.docx
(W5 block, now 23 features), WBS-Sprint-Plan.xlsx (W5 in register +
Sprint 3). Generated from updated markdown; consistency guard passed.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/exports/Nexorus-ATLAS-WBS-Sprint-Plan.xlsx
+++ b/docs/exports/Nexorus-ATLAS-WBS-Sprint-Plan.xlsx
@@ -15,7 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Feature Register'!$A$1:$G$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Feature Register'!$A$1:$G$24</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -568,7 +568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1027,27 +1027,27 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>U1</t>
+          <t>W5</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>LLM provider abstraction &amp; cost ledger</t>
-        </is>
-      </c>
-      <c r="C13" s="6" t="inlineStr">
-        <is>
-          <t>2-understand</t>
+          <t>Initial recent-window backfill</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>1-watch</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>S4</t>
+          <t>S3</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>E5</t>
+          <t>E4</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
@@ -1064,12 +1064,12 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>U2</t>
+          <t>U1</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Article enrichment (score/issues/sentiment/summary/keywords)</t>
+          <t>LLM provider abstraction &amp; cost ledger</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
@@ -1101,12 +1101,12 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>U3</t>
+          <t>U2</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Geocoding &amp; incident mapping</t>
+          <t>Article enrichment (score/issues/sentiment/summary/keywords)</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
@@ -1138,12 +1138,12 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>U4</t>
+          <t>U3</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Crisis snapshots &amp; trends</t>
+          <t>Geocoding &amp; incident mapping</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
@@ -1175,12 +1175,12 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>U5</t>
+          <t>U4</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Predictions, insights, actor &amp; leadership analytics</t>
+          <t>Crisis snapshots &amp; trends</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
@@ -1190,7 +1190,7 @@
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>S4-S5</t>
+          <t>S4</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
@@ -1212,27 +1212,27 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>A1</t>
+          <t>U5</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Dashboard read API &amp; caching</t>
-        </is>
-      </c>
-      <c r="C18" s="7" t="inlineStr">
-        <is>
-          <t>3-act</t>
+          <t>Predictions, insights, actor &amp; leadership analytics</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>2-understand</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>S2,S5</t>
+          <t>S4-S5</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>E6</t>
+          <t>E5</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
@@ -1249,12 +1249,12 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Widget integration &amp; live data</t>
+          <t>Dashboard read API &amp; caching</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
@@ -1264,7 +1264,7 @@
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>S5</t>
+          <t>S2,S5</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
@@ -1286,12 +1286,12 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>A3</t>
+          <t>A2</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Persisted dashboard layout</t>
+          <t>Widget integration &amp; live data</t>
         </is>
       </c>
       <c r="C20" s="7" t="inlineStr">
@@ -1323,12 +1323,12 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>A4</t>
+          <t>A3</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>AI assistant - copilot chat</t>
+          <t>Persisted dashboard layout</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
@@ -1343,7 +1343,7 @@
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>E7</t>
+          <t>E6</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
@@ -1360,12 +1360,12 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>A5</t>
+          <t>A4</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>AI assistant - briefing, forecast &amp; per-widget ask</t>
+          <t>AI assistant - copilot chat</t>
         </is>
       </c>
       <c r="C22" s="7" t="inlineStr">
@@ -1397,42 +1397,79 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
+          <t>A5</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>AI assistant - briefing, forecast &amp; per-widget ask</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>3-act</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>S5</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>E7</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
           <t>A6</t>
         </is>
       </c>
-      <c r="B23" s="3" t="inlineStr">
+      <c r="B24" s="3" t="inlineStr">
         <is>
           <t>Real-time ticker, alerts &amp; War Room</t>
         </is>
       </c>
-      <c r="C23" s="7" t="inlineStr">
+      <c r="C24" s="7" t="inlineStr">
         <is>
           <t>3-act</t>
         </is>
       </c>
-      <c r="D23" s="3" t="inlineStr">
+      <c r="D24" s="3" t="inlineStr">
         <is>
           <t>S5-S6</t>
         </is>
       </c>
-      <c r="E23" s="3" t="inlineStr">
+      <c r="E24" s="3" t="inlineStr">
         <is>
           <t>E8</t>
         </is>
       </c>
-      <c r="F23" s="3" t="inlineStr">
+      <c r="F24" s="3" t="inlineStr">
         <is>
           <t>1.0</t>
         </is>
       </c>
-      <c r="G23" s="3" t="inlineStr">
+      <c r="G24" s="3" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G23"/>
+  <autoFilter ref="A1:G24"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1547,7 +1584,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>W1, W2, W4, W3 (spike)</t>
+          <t>W1, W2, W4, W5, W3 (spike)</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">

</xml_diff>